<commit_message>
EPBDS-16529 Index a condition whose static check is joined by "and"
A condition such as "isNotEmpty(codes) and contains(codes, code)" was left to
the row by row evaluation, while the same check written with "or" was indexed.
The static answer now tells the index what to do: with "and" a true answer runs
the lookup and anything else leaves only the rules with an empty cell.
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
+++ b/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E127"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="3" max="3"/>
@@ -677,11 +677,10 @@
     <row r="28">
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>Rules String ContainsInInputArrayIndex_AfterEqualsIndex(String[] strs, String region)</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="2" t="n"/>
+          <t>Rules String ContainsInInputArrayIndex_WithStaticAnd(String[] strs)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="C29" s="3" t="inlineStr">
@@ -691,11 +690,6 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
           <t>RET1</t>
         </is>
       </c>
@@ -703,15 +697,10 @@
     <row r="30">
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>region == reg</t>
+          <t>isNotEmpty(strs) and contains(strs, val)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>contains(strs, val)</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>res</t>
         </is>
@@ -720,15 +709,10 @@
     <row r="31">
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>String reg</t>
+          <t>String val</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>String val</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>String res</t>
         </is>
@@ -737,15 +721,10 @@
     <row r="32">
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Region</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
@@ -754,24 +733,19 @@
     <row r="33">
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>foo</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
           <t>foo</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>EU-foo</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>bar</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -779,161 +753,157 @@
           <t>bar</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>EU-bar</t>
-        </is>
-      </c>
     </row>
     <row r="35">
-      <c r="C35" s="7" t="n"/>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>foo</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>ANY-foo</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>baz</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>ANY-baz</t>
-        </is>
-      </c>
-    </row>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
     <row r="37"/>
     <row r="38"/>
     <row r="39"/>
-    <row r="40"/>
+    <row r="40">
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_AfterEqualsIndex(String[] strs, String region)</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="2" t="n"/>
+    </row>
     <row r="41">
-      <c r="C41" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_BeforeRangeIndex(String[] strs, Integer amount)</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="2" t="n"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>RET1</t>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>region == reg</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>contains(strs, val)</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>contains(strs, val)</t>
+          <t>String reg</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>amount &gt;= minAmount</t>
+          <t>String val</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>res</t>
+          <t>String res</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>String val</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Integer minAmount</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>String res</t>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Min Amount</t>
+          <t>foo</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>EU-foo</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="C46" s="5" t="inlineStr">
         <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>EU-bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
           <t>foo</t>
         </is>
       </c>
-      <c r="D46" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>foo-100</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>foo</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="n">
-        <v>0</v>
-      </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>foo-0</t>
+          <t>ANY-foo</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>bar</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="n">
-        <v>0</v>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>baz</t>
+        </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>bar-0</t>
+          <t>ANY-baz</t>
         </is>
       </c>
     </row>
@@ -944,10 +914,11 @@
     <row r="53">
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t>Rules String ContainsInInputArrayIndex_WithCast(Integer[] amounts)</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="n"/>
+          <t>Rules String ContainsInInputArrayIndex_BeforeRangeIndex(String[] strs, Integer amount)</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="C54" s="3" t="inlineStr">
@@ -957,6 +928,11 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
           <t>RET1</t>
         </is>
       </c>
@@ -964,10 +940,15 @@
     <row r="55">
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>contains(amounts, amount)</t>
+          <t>contains(strs, val)</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>amount &gt;= minAmount</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>res</t>
         </is>
@@ -976,10 +957,15 @@
     <row r="56">
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Double amount</t>
+          <t>String val</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Integer minAmount</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>String res</t>
         </is>
@@ -988,514 +974,625 @@
     <row r="57">
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
+          <t>Min Amount</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
           <t>Result</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Ten</t>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>foo-100</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="C59" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Twenty</t>
-        </is>
-      </c>
-    </row>
-    <row r="60"/>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>foo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>bar-0</t>
+        </is>
+      </c>
+    </row>
     <row r="61"/>
     <row r="62"/>
     <row r="63"/>
-    <row r="64">
-      <c r="C64" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInArrayIndex_OppositeOrder(String str)</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="n"/>
-    </row>
+    <row r="64"/>
     <row r="65">
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_WithCast(Integer[] amounts)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>RET1</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>contains(vals, str)</t>
-        </is>
-      </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>res</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>String[] vals</t>
+          <t>contains(amounts, amount)</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Double amount</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
           <t>String res</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>Values</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>foo, bar</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>foo</t>
+          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>hello</t>
-        </is>
+      <c r="C70" s="5" t="n">
+        <v>10</v>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>hello</t>
-        </is>
-      </c>
-    </row>
-    <row r="71"/>
+          <t>Ten</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="C71" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Twenty</t>
+        </is>
+      </c>
+    </row>
     <row r="72"/>
     <row r="73"/>
     <row r="74"/>
-    <row r="75">
-      <c r="C75" s="1" t="inlineStr">
+    <row r="75"/>
+    <row r="76">
+      <c r="C76" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInArrayIndex_OppositeOrder(String str)</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>contains(vals, str)</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>String[] vals</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87">
+      <c r="C87" s="1" t="inlineStr">
         <is>
           <t>Datatype Coverage</t>
         </is>
       </c>
-      <c r="D75" s="2" t="n"/>
-    </row>
-    <row r="76">
-      <c r="C76" s="5" t="inlineStr">
+      <c r="D87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="C88" s="5" t="inlineStr">
         <is>
           <t>String[]</t>
         </is>
       </c>
-      <c r="D76" s="5" t="inlineStr">
+      <c r="D88" s="5" t="inlineStr">
         <is>
           <t>codes</t>
         </is>
       </c>
     </row>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81">
-      <c r="C81" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_WithPath(Coverage coverage)</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="n"/>
-    </row>
-    <row r="82">
-      <c r="C82" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>RET1</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>contains(coverage.codes, val)</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>res</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>String val</t>
-        </is>
-      </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>String res</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>foo</t>
-        </is>
-      </c>
-      <c r="D86" s="5" t="inlineStr">
-        <is>
-          <t>foo</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>bar</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>bar</t>
-        </is>
-      </c>
-    </row>
-    <row r="88"/>
     <row r="89"/>
     <row r="90"/>
     <row r="91"/>
-    <row r="92">
-      <c r="C92" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_PrimitiveArray(int[] ids)</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="n"/>
-    </row>
+    <row r="92"/>
     <row r="93">
-      <c r="C93" s="3" t="inlineStr">
+      <c r="C93" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_WithPath(Coverage coverage)</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="C94" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr">
+      <c r="D94" s="3" t="inlineStr">
         <is>
           <t>RET1</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>contains(ids, id)</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>res</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Integer id</t>
+          <t>contains(coverage.codes, val)</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>String val</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
           <t>String res</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>Id</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
+    <row r="97">
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="C97" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-    </row>
     <row r="98">
-      <c r="C98" s="5" t="n">
-        <v>2</v>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>two</t>
-        </is>
-      </c>
-    </row>
-    <row r="99"/>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+    </row>
     <row r="100"/>
     <row r="101"/>
     <row r="102"/>
-    <row r="103">
-      <c r="C103" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_WithDate(Date[] dates)</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="n"/>
-    </row>
+    <row r="103"/>
     <row r="104">
-      <c r="C104" s="3" t="inlineStr">
+      <c r="C104" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_PrimitiveArray(int[] ids)</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="C105" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="D104" s="3" t="inlineStr">
+      <c r="D105" s="3" t="inlineStr">
         <is>
           <t>RET1</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="C105" s="4" t="inlineStr">
-        <is>
-          <t>contains(dates, date)</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="inlineStr">
-        <is>
-          <t>res</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Date date</t>
+          <t>contains(ids, id)</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>Integer id</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
           <t>String res</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="C107" s="5" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D107" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>01/02/2020</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>first</t>
+          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="C109" s="5" t="inlineStr">
-        <is>
-          <t>03/04/2020</t>
-        </is>
+      <c r="C109" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>second</t>
-        </is>
-      </c>
-    </row>
-    <row r="110"/>
+          <t>one</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="C110" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>two</t>
+        </is>
+      </c>
+    </row>
     <row r="111"/>
     <row r="112"/>
     <row r="113"/>
-    <row r="114">
-      <c r="C114" s="1" t="inlineStr">
+    <row r="114"/>
+    <row r="115">
+      <c r="C115" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_WithDate(Date[] dates)</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="n"/>
+    </row>
+    <row r="116">
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>contains(dates, date)</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>Date date</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>01/02/2020</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>first</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>03/04/2020</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>second</t>
+        </is>
+      </c>
+    </row>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126">
+      <c r="C126" s="1" t="inlineStr">
         <is>
           <t>Datatype CoverageCode &lt;String&gt;</t>
         </is>
       </c>
-      <c r="D114" s="2" t="n"/>
-    </row>
-    <row r="115">
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>GADS</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="C116" s="5" t="inlineStr">
-        <is>
-          <t>GDHIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121">
-      <c r="C121" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_WithAlias(String[] codes)</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="n"/>
-    </row>
-    <row r="122">
-      <c r="C122" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="D122" s="3" t="inlineStr">
-        <is>
-          <t>RET1</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="C123" s="4" t="inlineStr">
-        <is>
-          <t>contains(codes, code)</t>
-        </is>
-      </c>
-      <c r="D123" s="4" t="inlineStr">
-        <is>
-          <t>res</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="C124" s="4" t="inlineStr">
-        <is>
-          <t>CoverageCode code</t>
-        </is>
-      </c>
-      <c r="D124" s="4" t="inlineStr">
-        <is>
-          <t>String res</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="C125" s="5" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="D125" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="C126" s="5" t="inlineStr">
-        <is>
-          <t>GADS</t>
-        </is>
-      </c>
-      <c r="D126" s="5" t="inlineStr">
-        <is>
-          <t>accident</t>
-        </is>
-      </c>
+      <c r="D126" s="2" t="n"/>
     </row>
     <row r="127">
       <c r="C127" s="5" t="inlineStr">
         <is>
+          <t>GADS</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="C128" s="5" t="inlineStr">
+        <is>
           <t>GDHIS</t>
         </is>
       </c>
-      <c r="D127" s="5" t="inlineStr">
+    </row>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133">
+      <c r="C133" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_WithAlias(String[] codes)</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="n"/>
+    </row>
+    <row r="134">
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>contains(codes, code)</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>CoverageCode code</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>GADS</t>
+        </is>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t>accident</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>GDHIS</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
         <is>
           <t>health</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C92:D92"/>
-    <mergeCell ref="C41:E41"/>
+  <mergeCells count="13">
     <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C103:D103"/>
-    <mergeCell ref="C81:D81"/>
-    <mergeCell ref="C121:D121"/>
-    <mergeCell ref="C75:D75"/>
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="C114:D114"/>
+    <mergeCell ref="C115:D115"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C104:D104"/>
+    <mergeCell ref="C76:D76"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="C93:D93"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C133:D133"/>
+    <mergeCell ref="C126:D126"/>
+    <mergeCell ref="C87:D87"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
EPBDS-16529 Index several lookups over the same array of inputs
A condition may ask for more than one column value in the same array, as
"contains(codes, code) or contains(codes, linkedCode)" does. Every such call
was left to the row by row evaluation, even though one index answers all of
them: the rule is registered under each of its values. The values may be
declared by another column of the table, which is how the customer tables
relate a coverage to its linked one.
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
+++ b/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E139"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="3" max="3"/>
@@ -773,7 +773,7 @@
     <row r="40">
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>Rules String ContainsInInputArrayIndex_AfterEqualsIndex(String[] strs, String region)</t>
+          <t>Rules String ContainsInInputArrayIndex_ChainOverColumns(String[] strs)</t>
         </is>
       </c>
       <c r="D40" s="6" t="n"/>
@@ -799,12 +799,12 @@
     <row r="42">
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>region == reg</t>
+          <t>isEmpty(strs) or contains(strs, val) or contains(strs, linkedVal)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>contains(strs, val)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -816,12 +816,12 @@
     <row r="43">
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>String reg</t>
+          <t>String val</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>String val</t>
+          <t>String linkedVal</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -833,12 +833,12 @@
     <row r="44">
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Region</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Linked Value</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -850,266 +850,301 @@
     <row r="45">
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>foo</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
+          <t>foo2</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
           <t>foo</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>EU-foo</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>bar</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
+          <t>bar2</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
           <t>bar</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>EU-bar</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="C47" s="7" t="n"/>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>foo</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>ANY-foo</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="C48" s="7" t="n"/>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>baz</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>ANY-baz</t>
-        </is>
-      </c>
-    </row>
+    </row>
+    <row r="47"/>
+    <row r="48"/>
     <row r="49"/>
     <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
+    <row r="51">
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_AfterEqualsIndex(String[] strs, String region)</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
     <row r="53">
-      <c r="C53" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_BeforeRangeIndex(String[] strs, Integer amount)</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="2" t="n"/>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>region == reg</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>contains(strs, val)</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>RET1</t>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>String reg</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>String val</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>contains(strs, val)</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>amount &gt;= minAmount</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>res</t>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>String val</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>Integer minAmount</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>String res</t>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>EU-foo</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Min Amount</t>
+          <t>bar</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>EU-bar</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C58" s="7" t="n"/>
+      <c r="D58" s="5" t="inlineStr">
         <is>
           <t>foo</t>
         </is>
       </c>
-      <c r="D58" s="5" t="n">
-        <v>100</v>
-      </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>foo-100</t>
+          <t>ANY-foo</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>foo</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="n">
-        <v>0</v>
+      <c r="C59" s="7" t="n"/>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>baz</t>
+        </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>foo-0</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>bar</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>bar-0</t>
-        </is>
-      </c>
-    </row>
+          <t>ANY-baz</t>
+        </is>
+      </c>
+    </row>
+    <row r="60"/>
     <row r="61"/>
     <row r="62"/>
     <row r="63"/>
-    <row r="64"/>
+    <row r="64">
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_BeforeRangeIndex(String[] strs, Integer amount)</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="2" t="n"/>
+    </row>
     <row r="65">
-      <c r="C65" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_WithCast(Integer[] amounts)</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="n"/>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>RET1</t>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>contains(strs, val)</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>amount &gt;= minAmount</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>contains(amounts, amount)</t>
+          <t>String val</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>res</t>
+          <t>Integer minAmount</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Double amount</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>String res</t>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Min Amount</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>foo-100</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="C70" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>Ten</t>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>foo-0</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="C71" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>Twenty</t>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>bar-0</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1155,7 @@
     <row r="76">
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>Rules String ContainsInArrayIndex_OppositeOrder(String str)</t>
+          <t>Rules String ContainsInInputArrayIndex_WithCast(Integer[] amounts)</t>
         </is>
       </c>
       <c r="D76" s="2" t="n"/>
@@ -1140,7 +1175,7 @@
     <row r="78">
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>contains(vals, str)</t>
+          <t>contains(amounts, amount)</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -1152,7 +1187,7 @@
     <row r="79">
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>String[] vals</t>
+          <t>Double amount</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -1164,7 +1199,7 @@
     <row r="80">
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Values</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
@@ -1174,26 +1209,22 @@
       </c>
     </row>
     <row r="81">
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>foo, bar</t>
-        </is>
+      <c r="C81" s="5" t="n">
+        <v>10</v>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>foo</t>
+          <t>Ten</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>hello</t>
-        </is>
+      <c r="C82" s="5" t="n">
+        <v>20</v>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>hello</t>
+          <t>Twenty</t>
         </is>
       </c>
     </row>
@@ -1204,104 +1235,104 @@
     <row r="87">
       <c r="C87" s="1" t="inlineStr">
         <is>
+          <t>Rules String ContainsInArrayIndex_OppositeOrder(String str)</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>contains(vals, str)</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>String[] vals</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98">
+      <c r="C98" s="1" t="inlineStr">
+        <is>
           <t>Datatype Coverage</t>
         </is>
       </c>
-      <c r="D87" s="2" t="n"/>
-    </row>
-    <row r="88">
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>String[]</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>codes</t>
-        </is>
-      </c>
-    </row>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93">
-      <c r="C93" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_WithPath(Coverage coverage)</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="n"/>
-    </row>
-    <row r="94">
-      <c r="C94" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="D94" s="3" t="inlineStr">
-        <is>
-          <t>RET1</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>contains(coverage.codes, val)</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>res</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="C96" s="4" t="inlineStr">
-        <is>
-          <t>String val</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>String res</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>foo</t>
-        </is>
-      </c>
-      <c r="D98" s="5" t="inlineStr">
-        <is>
-          <t>foo</t>
-        </is>
-      </c>
+      <c r="D98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>bar</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>bar</t>
+          <t>codes</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1343,7 @@
     <row r="104">
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>Rules String ContainsInInputArrayIndex_PrimitiveArray(int[] ids)</t>
+          <t>Rules String ContainsInInputArrayIndex_WithPath(Coverage coverage)</t>
         </is>
       </c>
       <c r="D104" s="2" t="n"/>
@@ -1332,7 +1363,7 @@
     <row r="106">
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>contains(ids, id)</t>
+          <t>contains(coverage.codes, val)</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -1344,7 +1375,7 @@
     <row r="107">
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Integer id</t>
+          <t>String val</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -1356,7 +1387,7 @@
     <row r="108">
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
@@ -1366,22 +1397,26 @@
       </c>
     </row>
     <row r="109">
-      <c r="C109" s="5" t="n">
-        <v>1</v>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>one</t>
+          <t>foo</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="C110" s="5" t="n">
-        <v>2</v>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>two</t>
+          <t>bar</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1427,7 @@
     <row r="115">
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>Rules String ContainsInInputArrayIndex_WithDate(Date[] dates)</t>
+          <t>Rules String ContainsInInputArrayIndex_PrimitiveArray(int[] ids)</t>
         </is>
       </c>
       <c r="D115" s="2" t="n"/>
@@ -1412,7 +1447,7 @@
     <row r="117">
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>contains(dates, date)</t>
+          <t>contains(ids, id)</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -1424,7 +1459,7 @@
     <row r="118">
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Date date</t>
+          <t>Integer id</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -1436,7 +1471,7 @@
     <row r="119">
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr">
@@ -1446,26 +1481,22 @@
       </c>
     </row>
     <row r="120">
-      <c r="C120" s="5" t="inlineStr">
-        <is>
-          <t>01/02/2020</t>
-        </is>
+      <c r="C120" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t>first</t>
+          <t>one</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="C121" s="5" t="inlineStr">
-        <is>
-          <t>03/04/2020</t>
-        </is>
+      <c r="C121" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t>second</t>
+          <t>two</t>
         </is>
       </c>
     </row>
@@ -1476,84 +1507,94 @@
     <row r="126">
       <c r="C126" s="1" t="inlineStr">
         <is>
+          <t>Rules String ContainsInInputArrayIndex_WithDate(Date[] dates)</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="n"/>
+    </row>
+    <row r="127">
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>contains(dates, date)</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>Date date</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>01/02/2020</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>first</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>03/04/2020</t>
+        </is>
+      </c>
+      <c r="D132" s="5" t="inlineStr">
+        <is>
+          <t>second</t>
+        </is>
+      </c>
+    </row>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137">
+      <c r="C137" s="1" t="inlineStr">
+        <is>
           <t>Datatype CoverageCode &lt;String&gt;</t>
         </is>
       </c>
-      <c r="D126" s="2" t="n"/>
-    </row>
-    <row r="127">
-      <c r="C127" s="5" t="inlineStr">
-        <is>
-          <t>GADS</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="C128" s="5" t="inlineStr">
-        <is>
-          <t>GDHIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133">
-      <c r="C133" s="1" t="inlineStr">
-        <is>
-          <t>Rules String ContainsInInputArrayIndex_WithAlias(String[] codes)</t>
-        </is>
-      </c>
-      <c r="D133" s="2" t="n"/>
-    </row>
-    <row r="134">
-      <c r="C134" s="3" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="D134" s="3" t="inlineStr">
-        <is>
-          <t>RET1</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="C135" s="4" t="inlineStr">
-        <is>
-          <t>contains(codes, code)</t>
-        </is>
-      </c>
-      <c r="D135" s="4" t="inlineStr">
-        <is>
-          <t>res</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="C136" s="4" t="inlineStr">
-        <is>
-          <t>CoverageCode code</t>
-        </is>
-      </c>
-      <c r="D136" s="4" t="inlineStr">
-        <is>
-          <t>String res</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="C137" s="5" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="D137" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
+      <c r="D137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="C138" s="5" t="inlineStr">
@@ -1561,11 +1602,6 @@
           <t>GADS</t>
         </is>
       </c>
-      <c r="D138" s="5" t="inlineStr">
-        <is>
-          <t>accident</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="C139" s="5" t="inlineStr">
@@ -1573,25 +1609,105 @@
           <t>GDHIS</t>
         </is>
       </c>
-      <c r="D139" s="5" t="inlineStr">
+    </row>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144">
+      <c r="C144" s="1" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_WithAlias(String[] codes)</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="n"/>
+    </row>
+    <row r="145">
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="C146" s="4" t="inlineStr">
+        <is>
+          <t>contains(codes, code)</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>CoverageCode code</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>GADS</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>accident</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>GDHIS</t>
+        </is>
+      </c>
+      <c r="D150" s="5" t="inlineStr">
         <is>
           <t>health</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
+    <mergeCell ref="C144:D144"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="C115:D115"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C98:D98"/>
+    <mergeCell ref="C76:D76"/>
     <mergeCell ref="C104:D104"/>
-    <mergeCell ref="C76:D76"/>
     <mergeCell ref="C40:E40"/>
-    <mergeCell ref="C93:D93"/>
+    <mergeCell ref="C137:D137"/>
     <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C133:D133"/>
+    <mergeCell ref="C64:E64"/>
     <mergeCell ref="C126:D126"/>
+    <mergeCell ref="C51:E51"/>
     <mergeCell ref="C87:D87"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>

</xml_diff>

<commit_message>
EPBDS-16529 Index a condition whose static check is written as a ternary
A condition such as "isNotEmpty(code) ? contains(codes, code) : fallback" was
left to the row by row evaluation, while the same check written with "or" or
"and" was indexed. The test now decides what the index does: true runs the
lookup, anything else answers the whole condition with the last part.

The test and the last part have to read the table inputs alone. A test that
reads the condition column answers differently from rule to rule, so such a
condition keeps the default evaluator.
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
+++ b/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
@@ -89,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -106,6 +106,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="C4:E172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="3" max="3"/>
@@ -479,9 +480,6 @@
     <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
     <row r="4">
       <c r="C4" s="1" t="inlineStr">
         <is>
@@ -574,10 +572,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16">
       <c r="C16" s="1" t="inlineStr">
         <is>
@@ -670,10 +664,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28">
       <c r="C28" s="1" t="inlineStr">
         <is>
@@ -766,10 +756,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40">
       <c r="C40" s="1" t="inlineStr">
         <is>
@@ -881,10 +867,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
     <row r="51">
       <c r="C51" s="1" t="inlineStr">
         <is>
@@ -1022,10 +1004,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
     <row r="64">
       <c r="C64" s="1" t="inlineStr">
         <is>
@@ -1148,10 +1126,6 @@
         </is>
       </c>
     </row>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
     <row r="76">
       <c r="C76" s="1" t="inlineStr">
         <is>
@@ -1228,10 +1202,6 @@
         </is>
       </c>
     </row>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
     <row r="87">
       <c r="C87" s="1" t="inlineStr">
         <is>
@@ -1312,10 +1282,6 @@
         </is>
       </c>
     </row>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
     <row r="98">
       <c r="C98" s="1" t="inlineStr">
         <is>
@@ -1336,10 +1302,6 @@
         </is>
       </c>
     </row>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
     <row r="104">
       <c r="C104" s="1" t="inlineStr">
         <is>
@@ -1420,10 +1382,6 @@
         </is>
       </c>
     </row>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
     <row r="115">
       <c r="C115" s="1" t="inlineStr">
         <is>
@@ -1500,10 +1458,6 @@
         </is>
       </c>
     </row>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
     <row r="126">
       <c r="C126" s="1" t="inlineStr">
         <is>
@@ -1584,10 +1538,6 @@
         </is>
       </c>
     </row>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
     <row r="137">
       <c r="C137" s="1" t="inlineStr">
         <is>
@@ -1610,10 +1560,6 @@
         </is>
       </c>
     </row>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
     <row r="144">
       <c r="C144" s="1" t="inlineStr">
         <is>
@@ -1691,6 +1637,164 @@
       <c r="D150" s="5" t="inlineStr">
         <is>
           <t>health</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInInputArrayIndex_WithTernary(String[] strs, Boolean fallback)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="C156" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="C157" s="7" t="inlineStr">
+        <is>
+          <t>isNotEmpty(strs) ? contains(strs, val) : fallback</t>
+        </is>
+      </c>
+      <c r="D157" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="C158" s="7" t="inlineStr">
+        <is>
+          <t>String val</t>
+        </is>
+      </c>
+      <c r="D158" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="C159" s="7" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D159" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="C160" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="D160" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="C161" s="7" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D161" s="7" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="C166" s="8" t="inlineStr">
+        <is>
+          <t>Rules String Ternary_TestOverColumn(String[] strs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="C167" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D167" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="C168" s="7" t="inlineStr">
+        <is>
+          <t>isNotEmpty(val) ? contains(strs, val) : true</t>
+        </is>
+      </c>
+      <c r="D168" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="C169" s="7" t="inlineStr">
+        <is>
+          <t>String val</t>
+        </is>
+      </c>
+      <c r="D169" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="C170" s="7" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D170" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="C171" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="D171" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="C172" s="7" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D172" s="7" t="inlineStr">
+        <is>
+          <t>bar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EPBDS-16529 Index a lookup guarded by a check that the column array is empty
A condition such as "isEmpty(codes) or contains(codes, code)" was evaluated row
by row. The check holds only for an empty cell, which matches anything in any
case, and the array of a filled cell always holds a value, so the whole
condition is the lookup alone.

The check has to name the very column the lookup searches, and isEmpty has to
be the built-in function rather than one the project declares.
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
+++ b/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C4:E172"/>
+  <dimension ref="C4:E183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="3" max="3"/>
@@ -1795,6 +1795,85 @@
       <c r="D172" s="7" t="inlineStr">
         <is>
           <t>bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="C177" s="8" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInArrayIndex_EmptyOrContains(String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="C178" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D178" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="C179" s="7" t="inlineStr">
+        <is>
+          <t>isEmpty(codes) or contains(codes, code)</t>
+        </is>
+      </c>
+      <c r="D179" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="C180" s="7" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="D180" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="C181" s="7" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="D181" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="C182" s="7" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D182" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="C183" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D183" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EPBDS-16529 Index a condition written as a call of a one-expression table
Projects hide the shapes the index understands behind a call of a helper table,
and such a condition was evaluated row by row. When the called table is written
of a single expression - a method table of one line, or a spreadsheet of one
step - that expression is read in the place of the call, with the arguments
written where the parameters stand, and the shapes are looked for inside it.

The expression may name its parameters and call the built-in functions, and
nothing else: a name of its own module is read again in the scope of the
decision table, where it may mean something else. A table that carries dimension
properties is not read this way either, because which of its versions answers a
call is decided at run time. The call itself is never replaced at run time, so
the rules the index does not answer are evaluated as before.
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
+++ b/STUDIO/org.openl.rules.webstudio/test/rules/decisionTableIndexes/EPBDS-16529.xlsx
@@ -43,7 +43,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -85,11 +85,12 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -107,6 +108,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="1" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -472,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C4:E183"/>
+  <dimension ref="C4:F288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="3" max="3"/>
@@ -1872,6 +1875,654 @@
         </is>
       </c>
       <c r="D183" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="C188" s="8" t="inlineStr">
+        <is>
+          <t>Constants</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="C189" s="7" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D189" s="7" t="inlineStr">
+        <is>
+          <t>DEFAULT_CODE</t>
+        </is>
+      </c>
+      <c r="E189" s="7" t="inlineStr">
+        <is>
+          <t>baz</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="C193" s="8" t="inlineStr">
+        <is>
+          <t>Method Boolean matchesCode(String[] codes, String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="C194" s="7" t="inlineStr">
+        <is>
+          <t>return isEmpty(codes) or contains(codes, code);</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="C198" s="8" t="inlineStr">
+        <is>
+          <t>Spreadsheet Boolean matchesDimension(String[] values, String value, Boolean fallback)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="C199" s="7" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="C200" s="7" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="D200" s="9" t="inlineStr">
+        <is>
+          <t>= isNotEmpty(value) ? isEmpty(values) or contains(values, value) : fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="C204" s="8" t="inlineStr">
+        <is>
+          <t>Method Boolean matchesInTwoLines(String[] codes, String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="C205" s="7" t="inlineStr">
+        <is>
+          <t>String wanted = code;</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="C206" s="7" t="inlineStr">
+        <is>
+          <t>return isEmpty(codes) or contains(codes, wanted);</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="C210" s="8" t="inlineStr">
+        <is>
+          <t>Method Boolean matchesDefault(String[] codes, String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="C211" s="7" t="inlineStr">
+        <is>
+          <t>return contains(codes, code) or contains(codes, DEFAULT_CODE);</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="C215" s="8" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInArrayIndex_ViaMethodTable(String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="C216" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D216" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="C217" s="7" t="inlineStr">
+        <is>
+          <t>matchesCode(codes, code)</t>
+        </is>
+      </c>
+      <c r="D217" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="C218" s="7" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="D218" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="C219" s="7" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="D219" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="C220" s="7" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D220" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="C221" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D221" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="C226" s="8" t="inlineStr">
+        <is>
+          <t>Rules String ContainsInArrayIndex_ViaSpreadsheet(String code, Boolean fallback)</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="C227" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D227" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="C228" s="7" t="inlineStr">
+        <is>
+          <t>matchesDimension(codes, code, fallback)</t>
+        </is>
+      </c>
+      <c r="D228" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="C229" s="7" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="D229" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="C230" s="7" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="D230" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="C231" s="7" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D231" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="C232" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D232" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="C237" s="8" t="inlineStr">
+        <is>
+          <t>Rules String Inline_TwoLineMethod(String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="C238" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D238" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="C239" s="7" t="inlineStr">
+        <is>
+          <t>matchesInTwoLines(codes, code)</t>
+        </is>
+      </c>
+      <c r="D239" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="C240" s="7" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="D240" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="C241" s="7" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="D241" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="C242" s="7" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D242" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="C243" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D243" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="C248" s="8" t="inlineStr">
+        <is>
+          <t>Rules String Inline_ModuleName(String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="C249" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D249" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="C250" s="7" t="inlineStr">
+        <is>
+          <t>matchesDefault(codes, code)</t>
+        </is>
+      </c>
+      <c r="D250" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="C251" s="7" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="D251" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="C252" s="7" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="D252" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="C253" s="7" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D253" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="C254" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D254" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="C259" s="8" t="inlineStr">
+        <is>
+          <t>Method Boolean matchesVersioned(String[] codes, String code)</t>
+        </is>
+      </c>
+      <c r="D259" s="8" t="n"/>
+      <c r="E259" s="8" t="n"/>
+      <c r="F259" s="10" t="n"/>
+    </row>
+    <row r="260">
+      <c r="C260" s="7" t="inlineStr">
+        <is>
+          <t>properties</t>
+        </is>
+      </c>
+      <c r="D260" s="7" t="inlineStr">
+        <is>
+          <t>effectiveDate</t>
+        </is>
+      </c>
+      <c r="E260" s="7" t="inlineStr">
+        <is>
+          <t>01/01/2020</t>
+        </is>
+      </c>
+      <c r="F260" s="10" t="n"/>
+    </row>
+    <row r="261">
+      <c r="C261" s="7" t="inlineStr">
+        <is>
+          <t>return isEmpty(codes) or contains(codes, code);</t>
+        </is>
+      </c>
+      <c r="D261" s="7" t="n"/>
+      <c r="E261" s="7" t="n"/>
+      <c r="F261" s="10" t="n"/>
+    </row>
+    <row r="262">
+      <c r="C262" s="10" t="n"/>
+      <c r="D262" s="10" t="n"/>
+      <c r="E262" s="10" t="n"/>
+      <c r="F262" s="10" t="n"/>
+    </row>
+    <row r="263">
+      <c r="C263" s="10" t="n"/>
+      <c r="D263" s="10" t="n"/>
+      <c r="E263" s="10" t="n"/>
+      <c r="F263" s="10" t="n"/>
+    </row>
+    <row r="264">
+      <c r="C264" s="10" t="n"/>
+      <c r="D264" s="10" t="n"/>
+      <c r="E264" s="10" t="n"/>
+      <c r="F264" s="10" t="n"/>
+    </row>
+    <row r="266">
+      <c r="C266" s="8" t="inlineStr">
+        <is>
+          <t>Method Boolean matchesViaTable(String[] codes, String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="C267" s="7" t="inlineStr">
+        <is>
+          <t>return matchesCode(codes, code);</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="C271" s="8" t="inlineStr">
+        <is>
+          <t>Rules String Inline_VersionedTable(String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="C272" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D272" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="C273" s="7" t="inlineStr">
+        <is>
+          <t>matchesVersioned(codes, code)</t>
+        </is>
+      </c>
+      <c r="D273" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="C274" s="7" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="D274" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="C275" s="7" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="D275" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="C276" s="7" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D276" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="C277" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D277" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="C282" s="8" t="inlineStr">
+        <is>
+          <t>Rules String Inline_CallOfAnotherTable(String code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="C283" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D283" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="C284" s="7" t="inlineStr">
+        <is>
+          <t>matchesViaTable(codes, code)</t>
+        </is>
+      </c>
+      <c r="D284" s="7" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="C285" s="7" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="D285" s="7" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="C286" s="7" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="D286" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="C287" s="7" t="inlineStr">
+        <is>
+          <t>foo, bar</t>
+        </is>
+      </c>
+      <c r="D287" s="7" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="C288" s="7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D288" s="7" t="inlineStr">
         <is>
           <t>hello</t>
         </is>

</xml_diff>